<commit_message>
RelatoriosService enviando o faturamento
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_baixo_estoque.xlsx
+++ b/relatorios/relatorio_baixo_estoque.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -29,6 +29,12 @@
     <t>Situação</t>
   </si>
   <si>
+    <t>Ryzen 5 5600</t>
+  </si>
+  <si>
+    <t>CRÍTICO</t>
+  </si>
+  <si>
     <t>Intel i7-12700K</t>
   </si>
   <si>
@@ -41,15 +47,15 @@
     <t>Core i5-13600K</t>
   </si>
   <si>
-    <t>CRÍTICO</t>
-  </si>
-  <si>
     <t>B550M Aorus Elite</t>
   </si>
   <si>
     <t>X670E ASUS ROG</t>
   </si>
   <si>
+    <t>H610M-E</t>
+  </si>
+  <si>
     <t>Z790 MSI Pro</t>
   </si>
   <si>
@@ -69,12 +75,6 @@
   </si>
   <si>
     <t>RX 6750 XT</t>
-  </si>
-  <si>
-    <t>Ryzen 5 5600</t>
-  </si>
-  <si>
-    <t>H610M-E</t>
   </si>
   <si>
     <t>RTX 3060</t>
@@ -160,7 +160,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="3.9296875" customWidth="true" bestFit="true"/>
@@ -189,24 +189,24 @@
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>5</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="D2" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E2" t="s" s="2">
+      <c r="E2" t="s" s="0">
         <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>7</v>
@@ -218,63 +218,63 @@
         <v>10.0</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C4" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D4" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="E4" t="s" s="2">
         <v>8</v>
-      </c>
-      <c r="C4" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="D4" t="n" s="0">
-        <v>10.0</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n" s="0">
-        <v>6.0</v>
+        <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>10</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="D5" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E5" t="s" s="2">
+      <c r="E5" t="s" s="0">
         <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n" s="0">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>11</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D6" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E6" t="s" s="0">
-        <v>9</v>
+      <c r="E6" t="s" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n" s="0">
-        <v>10.0</v>
+        <v>7.0</v>
       </c>
       <c r="B7" t="s" s="0">
         <v>12</v>
@@ -286,270 +286,270 @@
         <v>10.0</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n" s="0">
-        <v>12.0</v>
+        <v>8.0</v>
       </c>
       <c r="B8" t="s" s="0">
         <v>13</v>
       </c>
       <c r="C8" t="n" s="0">
-        <v>4.0</v>
+        <v>10.0</v>
       </c>
       <c r="D8" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n" s="0">
-        <v>15.0</v>
+        <v>10.0</v>
       </c>
       <c r="B9" t="s" s="0">
         <v>14</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>7.0</v>
+        <v>0.0</v>
       </c>
       <c r="D9" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E9" t="s" s="0">
-        <v>9</v>
+      <c r="E9" t="s" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n" s="0">
-        <v>16.0</v>
+        <v>12.0</v>
       </c>
       <c r="B10" t="s" s="0">
         <v>15</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="D10" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E10" t="s" s="2">
+      <c r="E10" t="s" s="0">
         <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
       <c r="B11" t="s" s="0">
         <v>16</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>1.0</v>
+        <v>9.0</v>
       </c>
       <c r="D11" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n" s="0">
-        <v>19.0</v>
+        <v>16.0</v>
       </c>
       <c r="B12" t="s" s="0">
         <v>17</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>6.0</v>
+        <v>0.0</v>
       </c>
       <c r="D12" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E12" t="s" s="0">
-        <v>9</v>
+      <c r="E12" t="s" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n" s="0">
-        <v>20.0</v>
+        <v>18.0</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>18</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="D13" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E13" t="s" s="0">
-        <v>9</v>
+      <c r="E13" t="s" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n" s="0">
-        <v>22.0</v>
+        <v>19.0</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>19</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>9.0</v>
+        <v>5.0</v>
       </c>
       <c r="D14" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n" s="0">
-        <v>23.0</v>
+        <v>20.0</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="D15" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E15" t="s" s="0">
-        <v>9</v>
+      <c r="E15" t="s" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n" s="0">
-        <v>24.0</v>
+        <v>21.0</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>3.0</v>
+        <v>10.0</v>
       </c>
       <c r="D16" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n" s="0">
-        <v>25.0</v>
+        <v>22.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>7.0</v>
+        <v>9.0</v>
       </c>
       <c r="D17" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n" s="0">
-        <v>27.0</v>
+        <v>23.0</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>7.0</v>
+        <v>5.0</v>
       </c>
       <c r="D18" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n" s="0">
-        <v>28.0</v>
+        <v>24.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D19" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n" s="0">
-        <v>29.0</v>
+        <v>25.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>10.0</v>
+        <v>7.0</v>
       </c>
       <c r="D20" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n" s="0">
-        <v>31.0</v>
+        <v>27.0</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="D21" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E21" t="s" s="2">
+      <c r="E21" t="s" s="0">
         <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n" s="0">
-        <v>33.0</v>
+        <v>28.0</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="D22" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n" s="0">
-        <v>37.0</v>
+        <v>29.0</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C23" t="n" s="0">
         <v>10.0</v>
@@ -558,100 +558,100 @@
         <v>10.0</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n" s="0">
-        <v>39.0</v>
+        <v>31.0</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="D24" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n" s="0">
-        <v>40.0</v>
+        <v>33.0</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>7.0</v>
+        <v>0.0</v>
       </c>
       <c r="D25" t="n" s="0">
         <v>10.0</v>
       </c>
-      <c r="E25" t="s" s="0">
-        <v>9</v>
+      <c r="E25" t="s" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n" s="0">
-        <v>41.0</v>
+        <v>37.0</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>5.0</v>
+        <v>10.0</v>
       </c>
       <c r="D26" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n" s="0">
-        <v>42.0</v>
+        <v>39.0</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>10.0</v>
+        <v>5.0</v>
       </c>
       <c r="D27" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n" s="0">
-        <v>139.0</v>
+        <v>40.0</v>
       </c>
       <c r="B28" t="s" s="0">
         <v>19</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>10.0</v>
+        <v>7.0</v>
       </c>
       <c r="D28" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n" s="0">
-        <v>140.0</v>
+        <v>41.0</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C29" t="n" s="0">
         <v>5.0</v>
@@ -660,177 +660,228 @@
         <v>10.0</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n" s="0">
-        <v>141.0</v>
+        <v>42.0</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>3.0</v>
+        <v>10.0</v>
       </c>
       <c r="D30" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n" s="0">
-        <v>142.0</v>
+        <v>139.0</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>8.0</v>
+        <v>10.0</v>
       </c>
       <c r="D31" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n" s="0">
-        <v>144.0</v>
+        <v>140.0</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>8.0</v>
+        <v>5.0</v>
       </c>
       <c r="D32" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n" s="0">
-        <v>145.0</v>
+        <v>141.0</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C33" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D33" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n" s="0">
-        <v>148.0</v>
+        <v>142.0</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C34" t="n" s="0">
-        <v>6.0</v>
+        <v>8.0</v>
       </c>
       <c r="D34" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n" s="0">
-        <v>150.0</v>
+        <v>144.0</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C35" t="n" s="0">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
       <c r="D35" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n" s="0">
-        <v>154.0</v>
+        <v>145.0</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C36" t="n" s="0">
-        <v>10.0</v>
+        <v>4.0</v>
       </c>
       <c r="D36" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n" s="0">
-        <v>156.0</v>
+        <v>148.0</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C37" t="n" s="0">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="D37" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n" s="0">
-        <v>157.0</v>
+        <v>150.0</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C38" t="n" s="0">
-        <v>7.0</v>
+        <v>10.0</v>
       </c>
       <c r="D38" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n" s="0">
+        <v>154.0</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C39" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="D39" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="E39" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n" s="0">
+        <v>156.0</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C40" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="D40" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="E40" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n" s="0">
+        <v>157.0</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C41" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="D41" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="E41" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n" s="0">
         <v>158.0</v>
       </c>
-      <c r="B39" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="C39" t="n" s="0">
+      <c r="B42" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C42" t="n" s="0">
         <v>5.0</v>
       </c>
-      <c r="D39" t="n" s="0">
-        <v>10.0</v>
-      </c>
-      <c r="E39" t="s" s="0">
-        <v>9</v>
+      <c r="D42" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="E42" t="s" s="0">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>